<commit_message>
fixed coop ui bug
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/dev/Relics.xlsx
+++ b/Assets/StreamingAssets/Configurations/dev/Relics.xlsx
@@ -1,16 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\dev\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B87ADEB7-BA19-468A-A531-4F11D3E00C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="10480" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RaisingRelicConditions" sheetId="1" r:id="rId1"/>
     <sheet name="Relics" sheetId="2" r:id="rId2"/>
     <sheet name="Consumables" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Relics!$A$1:$R$47</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -626,361 +635,25 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="20">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -997,315 +670,28 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1563,22 +949,22 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.18333333333333" customWidth="1"/>
-    <col min="2" max="2" width="11.725" customWidth="1"/>
-    <col min="3" max="3" width="15.45" customWidth="1"/>
-    <col min="4" max="4" width="28.725" customWidth="1"/>
-    <col min="5" max="5" width="14.725" customWidth="1"/>
-    <col min="6" max="6" width="13.45" customWidth="1"/>
-    <col min="7" max="7" width="10.45" customWidth="1"/>
+    <col min="1" max="1" width="3.140625" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1764,7 +1150,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" customFormat="1" spans="1:7">
+    <row r="10" spans="1:7">
       <c r="A10">
         <v>8</v>
       </c>
@@ -1784,7 +1170,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" customFormat="1" spans="1:7">
+    <row r="11" spans="1:7">
       <c r="A11">
         <v>9</v>
       </c>
@@ -1804,7 +1190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" customFormat="1" spans="1:7">
+    <row r="12" spans="1:7">
       <c r="A12">
         <v>10</v>
       </c>
@@ -1824,7 +1210,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" customFormat="1" spans="1:7">
+    <row r="13" spans="1:7">
       <c r="A13">
         <v>11</v>
       </c>
@@ -1886,36 +1272,34 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R47"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.41666666666667" customWidth="1"/>
-    <col min="2" max="2" width="13.5416666666667" customWidth="1"/>
-    <col min="3" max="3" width="25.45" customWidth="1"/>
-    <col min="4" max="4" width="12.1833333333333" customWidth="1"/>
-    <col min="5" max="5" width="5.45" customWidth="1"/>
-    <col min="6" max="6" width="20.1833333333333" customWidth="1"/>
-    <col min="7" max="7" width="3.81666666666667" customWidth="1"/>
-    <col min="8" max="8" width="7.45" customWidth="1"/>
-    <col min="9" max="9" width="10.2666666666667" customWidth="1"/>
-    <col min="10" max="10" width="13.1833333333333" customWidth="1"/>
-    <col min="11" max="11" width="17.1833333333333" customWidth="1"/>
-    <col min="12" max="12" width="14.1833333333333" customWidth="1"/>
-    <col min="13" max="13" width="12.45" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" customWidth="1"/>
+    <col min="3" max="3" width="25.42578125" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" customWidth="1"/>
+    <col min="5" max="5" width="5.42578125" customWidth="1"/>
+    <col min="6" max="6" width="20.140625" customWidth="1"/>
+    <col min="7" max="7" width="3.85546875" customWidth="1"/>
+    <col min="8" max="8" width="7.42578125" customWidth="1"/>
+    <col min="9" max="9" width="10.28515625" customWidth="1"/>
+    <col min="10" max="10" width="13.140625" customWidth="1"/>
+    <col min="11" max="11" width="17.140625" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" customWidth="1"/>
+    <col min="13" max="13" width="12.42578125" customWidth="1"/>
     <col min="14" max="14" width="17" customWidth="1"/>
-    <col min="15" max="15" width="11.8166666666667" customWidth="1"/>
-    <col min="16" max="16" width="11.5416666666667" customWidth="1"/>
-    <col min="17" max="17" width="17.1833333333333" customWidth="1"/>
+    <col min="15" max="15" width="11.85546875" customWidth="1"/>
+    <col min="16" max="16" width="11.5703125" customWidth="1"/>
+    <col min="17" max="17" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" spans="1:18">
+    <row r="1" spans="1:18" ht="30">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1971,7 +1355,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:18">
       <c r="A2">
         <v>0</v>
       </c>
@@ -2003,7 +1387,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:18">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2035,7 +1419,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:18">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2067,7 +1451,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:18">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2099,7 +1483,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:18">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2131,7 +1515,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:18">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2163,7 +1547,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:18">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2195,7 +1579,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:18">
       <c r="A9">
         <v>7</v>
       </c>
@@ -2227,7 +1611,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:18">
       <c r="A10">
         <v>8</v>
       </c>
@@ -2259,7 +1643,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:18">
       <c r="A11">
         <v>9</v>
       </c>
@@ -2291,7 +1675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:18">
       <c r="A12">
         <v>10</v>
       </c>
@@ -2320,7 +1704,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:18">
       <c r="A13">
         <v>11</v>
       </c>
@@ -2349,7 +1733,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:18">
       <c r="A14">
         <v>12</v>
       </c>
@@ -2375,7 +1759,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:18">
       <c r="A15">
         <v>13</v>
       </c>
@@ -2401,7 +1785,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:18">
       <c r="A16">
         <v>14</v>
       </c>
@@ -2870,7 +2254,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="33" spans="1:10">
+    <row r="33" spans="1:14">
       <c r="A33">
         <v>31</v>
       </c>
@@ -2899,7 +2283,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="34" spans="1:10">
+    <row r="34" spans="1:14">
       <c r="A34">
         <v>32</v>
       </c>
@@ -2928,7 +2312,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="35" spans="1:10">
+    <row r="35" spans="1:14">
       <c r="A35">
         <v>33</v>
       </c>
@@ -2954,7 +2338,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="36" spans="1:10">
+    <row r="36" spans="1:14">
       <c r="A36">
         <v>34</v>
       </c>
@@ -2980,7 +2364,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="37" spans="1:10">
+    <row r="37" spans="1:14">
       <c r="A37">
         <v>35</v>
       </c>
@@ -3006,7 +2390,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="38" spans="1:10">
+    <row r="38" spans="1:14">
       <c r="A38">
         <v>36</v>
       </c>
@@ -3032,7 +2416,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="39" spans="1:10">
+    <row r="39" spans="1:14">
       <c r="A39">
         <v>37</v>
       </c>
@@ -3058,7 +2442,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="40" spans="1:10">
+    <row r="40" spans="1:14">
       <c r="A40">
         <v>38</v>
       </c>
@@ -3084,7 +2468,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="41" spans="1:10">
+    <row r="41" spans="1:14">
       <c r="A41">
         <v>39</v>
       </c>
@@ -3113,7 +2497,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:10">
+    <row r="42" spans="1:14">
       <c r="A42">
         <v>40</v>
       </c>
@@ -3142,7 +2526,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:10">
+    <row r="43" spans="1:14">
       <c r="A43">
         <v>41</v>
       </c>
@@ -3171,7 +2555,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:10">
+    <row r="44" spans="1:14">
       <c r="A44">
         <v>42</v>
       </c>
@@ -3197,7 +2581,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:10">
+    <row r="45" spans="1:14">
       <c r="A45">
         <v>43</v>
       </c>
@@ -3223,7 +2607,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:10">
+    <row r="46" spans="1:14">
       <c r="A46">
         <v>44</v>
       </c>
@@ -3285,25 +2669,24 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:R47" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M14"/>
-  <sheetFormatPr defaultColWidth="8.725" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="23.5416666666667" customWidth="1"/>
-    <col min="4" max="7" width="18.1833333333333" customWidth="1"/>
-    <col min="8" max="8" width="10.5416666666667" customWidth="1"/>
+    <col min="3" max="3" width="23.5703125" customWidth="1"/>
+    <col min="4" max="7" width="18.140625" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="12.8166666666667" customWidth="1"/>
+    <col min="10" max="10" width="12.85546875" customWidth="1"/>
     <col min="11" max="11" width="11" customWidth="1"/>
-    <col min="12" max="12" width="11.2666666666667" customWidth="1"/>
-    <col min="13" max="13" width="10.725" customWidth="1"/>
+    <col min="12" max="12" width="11.28515625" customWidth="1"/>
+    <col min="13" max="13" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -3347,7 +2730,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:13">
       <c r="A2">
         <v>0</v>
       </c>
@@ -3376,7 +2759,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:13">
       <c r="A3">
         <v>1</v>
       </c>
@@ -3405,7 +2788,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:13">
       <c r="A4">
         <v>2</v>
       </c>
@@ -3434,7 +2817,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:13">
       <c r="A5">
         <v>3</v>
       </c>
@@ -3463,7 +2846,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:13">
       <c r="A6">
         <v>4</v>
       </c>
@@ -3492,7 +2875,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" ht="42" spans="1:13">
+    <row r="7" spans="1:13" ht="60">
       <c r="A7">
         <v>5</v>
       </c>
@@ -3533,7 +2916,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" ht="28" spans="1:10">
+    <row r="8" spans="1:13" ht="30">
       <c r="A8">
         <v>6</v>
       </c>
@@ -3565,7 +2948,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" ht="42" spans="1:11">
+    <row r="9" spans="1:13" ht="45">
       <c r="A9">
         <v>7</v>
       </c>
@@ -3600,7 +2983,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:13">
       <c r="A10">
         <v>8</v>
       </c>
@@ -3632,7 +3015,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:13">
       <c r="A11">
         <v>9</v>
       </c>
@@ -3667,7 +3050,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:13">
       <c r="A12">
         <v>10</v>
       </c>
@@ -3696,7 +3079,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:13">
       <c r="A13">
         <v>11</v>
       </c>
@@ -3725,12 +3108,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="6:7">
+    <row r="14" spans="1:13">
       <c r="F14" s="1"/>
-      <c r="G14" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Raising Animation System 3
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/dev/Relics.xlsx
+++ b/Assets/StreamingAssets/Configurations/dev/Relics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E32FD38E-6640-4347-8795-0E7CAFE8CA7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF62DF9E-BF47-4A51-BE08-207481F17081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -425,9 +425,6 @@
     <t>每阶段结束时，获得粉丝数1%的歌力</t>
   </si>
   <si>
-    <t>OnPhaseEndingSelected</t>
-  </si>
-  <si>
     <t>粉丝徽章-游戏区</t>
   </si>
   <si>
@@ -628,18 +625,28 @@
   </si>
   <si>
     <t>drink11</t>
+  </si>
+  <si>
+    <t>OnPhaseEnd</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -672,12 +679,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1275,6 +1283,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:R47"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
@@ -1284,7 +1293,7 @@
     <col min="4" max="4" width="12.140625" customWidth="1"/>
     <col min="5" max="5" width="5.42578125" customWidth="1"/>
     <col min="6" max="6" width="20.140625" customWidth="1"/>
-    <col min="7" max="7" width="3.85546875" customWidth="1"/>
+    <col min="7" max="7" width="6.140625" customWidth="1"/>
     <col min="8" max="8" width="7.42578125" customWidth="1"/>
     <col min="9" max="9" width="10.28515625" customWidth="1"/>
     <col min="10" max="10" width="13.140625" customWidth="1"/>
@@ -1297,7 +1306,7 @@
     <col min="17" max="17" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="30">
+    <row r="1" spans="1:18">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1702,7 +1711,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="13" spans="1:18">
+    <row r="13" spans="1:18" hidden="1">
       <c r="A13">
         <v>11</v>
       </c>
@@ -1718,7 +1727,7 @@
       <c r="E13">
         <v>3</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="3" t="s">
         <v>71</v>
       </c>
       <c r="I13">
@@ -1809,7 +1818,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" hidden="1">
       <c r="A17">
         <v>15</v>
       </c>
@@ -1835,7 +1844,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" hidden="1">
       <c r="A18">
         <v>16</v>
       </c>
@@ -1861,7 +1870,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" hidden="1">
       <c r="A19">
         <v>17</v>
       </c>
@@ -1991,7 +2000,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" hidden="1">
       <c r="A24">
         <v>22</v>
       </c>
@@ -2020,7 +2029,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" hidden="1">
       <c r="A25">
         <v>23</v>
       </c>
@@ -2049,7 +2058,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" hidden="1">
       <c r="A26">
         <v>24</v>
       </c>
@@ -2078,7 +2087,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" hidden="1">
       <c r="A27">
         <v>25</v>
       </c>
@@ -2223,7 +2232,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" hidden="1">
       <c r="A32">
         <v>30</v>
       </c>
@@ -2252,7 +2261,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="33" spans="1:14">
+    <row r="33" spans="1:14" hidden="1">
       <c r="A33">
         <v>31</v>
       </c>
@@ -2281,7 +2290,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="34" spans="1:14">
+    <row r="34" spans="1:14" hidden="1">
       <c r="A34">
         <v>32</v>
       </c>
@@ -2326,7 +2335,7 @@
       <c r="E35">
         <v>-1</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F35" s="3" t="s">
         <v>122</v>
       </c>
       <c r="I35">
@@ -2395,7 +2404,7 @@
       <c r="B38" t="s">
         <v>127</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="3" t="s">
         <v>128</v>
       </c>
       <c r="D38" t="s">
@@ -2404,8 +2413,8 @@
       <c r="E38">
         <v>-1</v>
       </c>
-      <c r="F38" t="s">
-        <v>129</v>
+      <c r="F38" s="3" t="s">
+        <v>195</v>
       </c>
       <c r="I38">
         <v>60</v>
@@ -2419,19 +2428,19 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
+        <v>129</v>
+      </c>
+      <c r="C39" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="C39" t="s">
-        <v>131</v>
-      </c>
       <c r="D39" t="s">
         <v>45</v>
       </c>
       <c r="E39">
         <v>-1</v>
       </c>
-      <c r="F39" t="s">
-        <v>129</v>
+      <c r="F39" s="3" t="s">
+        <v>195</v>
       </c>
       <c r="I39">
         <v>61</v>
@@ -2445,19 +2454,19 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
+        <v>131</v>
+      </c>
+      <c r="C40" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="C40" t="s">
-        <v>133</v>
-      </c>
       <c r="D40" t="s">
         <v>45</v>
       </c>
       <c r="E40">
         <v>-1</v>
       </c>
-      <c r="F40" t="s">
-        <v>129</v>
+      <c r="F40" s="3" t="s">
+        <v>195</v>
       </c>
       <c r="I40">
         <v>62</v>
@@ -2471,19 +2480,19 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
+        <v>133</v>
+      </c>
+      <c r="C41" t="s">
         <v>134</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
+        <v>45</v>
+      </c>
+      <c r="E41">
+        <v>-1</v>
+      </c>
+      <c r="F41" t="s">
         <v>135</v>
-      </c>
-      <c r="D41" t="s">
-        <v>45</v>
-      </c>
-      <c r="E41">
-        <v>-1</v>
-      </c>
-      <c r="F41" t="s">
-        <v>136</v>
       </c>
       <c r="H41">
         <v>12</v>
@@ -2500,11 +2509,11 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
+        <v>136</v>
+      </c>
+      <c r="C42" t="s">
         <v>137</v>
       </c>
-      <c r="C42" t="s">
-        <v>138</v>
-      </c>
       <c r="D42" t="s">
         <v>45</v>
       </c>
@@ -2512,7 +2521,7 @@
         <v>-1</v>
       </c>
       <c r="F42" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H42">
         <v>12</v>
@@ -2529,11 +2538,11 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
+        <v>138</v>
+      </c>
+      <c r="C43" t="s">
         <v>139</v>
       </c>
-      <c r="C43" t="s">
-        <v>140</v>
-      </c>
       <c r="D43" t="s">
         <v>45</v>
       </c>
@@ -2541,7 +2550,7 @@
         <v>-1</v>
       </c>
       <c r="F43" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H43">
         <v>12</v>
@@ -2558,19 +2567,19 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
+        <v>140</v>
+      </c>
+      <c r="C44" t="s">
         <v>141</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
+        <v>45</v>
+      </c>
+      <c r="E44">
+        <v>-1</v>
+      </c>
+      <c r="F44" t="s">
         <v>142</v>
-      </c>
-      <c r="D44" t="s">
-        <v>45</v>
-      </c>
-      <c r="E44">
-        <v>-1</v>
-      </c>
-      <c r="F44" t="s">
-        <v>143</v>
       </c>
       <c r="I44">
         <v>28</v>
@@ -2584,11 +2593,11 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
+        <v>143</v>
+      </c>
+      <c r="C45" t="s">
         <v>144</v>
       </c>
-      <c r="C45" t="s">
-        <v>145</v>
-      </c>
       <c r="D45" t="s">
         <v>45</v>
       </c>
@@ -2596,7 +2605,7 @@
         <v>-1</v>
       </c>
       <c r="F45" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I45">
         <v>29</v>
@@ -2610,11 +2619,11 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
+        <v>145</v>
+      </c>
+      <c r="C46" t="s">
         <v>146</v>
       </c>
-      <c r="C46" t="s">
-        <v>147</v>
-      </c>
       <c r="D46" t="s">
         <v>45</v>
       </c>
@@ -2622,7 +2631,7 @@
         <v>-1</v>
       </c>
       <c r="F46" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I46">
         <v>30</v>
@@ -2636,19 +2645,19 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
+        <v>147</v>
+      </c>
+      <c r="C47" t="s">
         <v>148</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
+        <v>45</v>
+      </c>
+      <c r="E47">
+        <v>-1</v>
+      </c>
+      <c r="F47" t="s">
         <v>149</v>
-      </c>
-      <c r="D47" t="s">
-        <v>45</v>
-      </c>
-      <c r="E47">
-        <v>-1</v>
-      </c>
-      <c r="F47" t="s">
-        <v>150</v>
       </c>
       <c r="I47">
         <v>15</v>
@@ -2667,7 +2676,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R47" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A1:R47" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="VRaisingRelic"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2701,10 +2716,10 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F1" t="s">
         <v>151</v>
-      </c>
-      <c r="F1" t="s">
-        <v>152</v>
       </c>
       <c r="G1" t="s">
         <v>42</v>
@@ -2733,22 +2748,22 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C2" t="s">
         <v>153</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>154</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>155</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>156</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>157</v>
-      </c>
-      <c r="G2" t="s">
-        <v>158</v>
       </c>
       <c r="H2">
         <v>3</v>
@@ -2762,22 +2777,22 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C3" t="s">
         <v>159</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E3" t="s">
         <v>160</v>
       </c>
-      <c r="D3" t="s">
-        <v>155</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
+        <v>156</v>
+      </c>
+      <c r="G3" t="s">
         <v>161</v>
-      </c>
-      <c r="F3" t="s">
-        <v>157</v>
-      </c>
-      <c r="G3" t="s">
-        <v>162</v>
       </c>
       <c r="H3">
         <v>15</v>
@@ -2791,22 +2806,22 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>162</v>
+      </c>
+      <c r="C4" t="s">
         <v>163</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E4" t="s">
+        <v>160</v>
+      </c>
+      <c r="F4" t="s">
+        <v>156</v>
+      </c>
+      <c r="G4" t="s">
         <v>164</v>
-      </c>
-      <c r="D4" t="s">
-        <v>155</v>
-      </c>
-      <c r="E4" t="s">
-        <v>161</v>
-      </c>
-      <c r="F4" t="s">
-        <v>157</v>
-      </c>
-      <c r="G4" t="s">
-        <v>165</v>
       </c>
       <c r="H4">
         <v>45</v>
@@ -2820,22 +2835,22 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>165</v>
+      </c>
+      <c r="C5" t="s">
         <v>166</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E5" t="s">
+        <v>155</v>
+      </c>
+      <c r="F5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G5" t="s">
         <v>167</v>
-      </c>
-      <c r="D5" t="s">
-        <v>155</v>
-      </c>
-      <c r="E5" t="s">
-        <v>156</v>
-      </c>
-      <c r="F5" t="s">
-        <v>157</v>
-      </c>
-      <c r="G5" t="s">
-        <v>168</v>
       </c>
       <c r="H5">
         <v>11</v>
@@ -2849,22 +2864,22 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>168</v>
+      </c>
+      <c r="C6" t="s">
         <v>169</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>170</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
+        <v>155</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="E6" t="s">
-        <v>156</v>
-      </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" t="s">
         <v>172</v>
-      </c>
-      <c r="G6" t="s">
-        <v>173</v>
       </c>
       <c r="H6">
         <v>38</v>
@@ -2878,22 +2893,22 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>173</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" t="s">
+        <v>154</v>
+      </c>
+      <c r="E7" t="s">
+        <v>155</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="G7" t="s">
         <v>175</v>
-      </c>
-      <c r="D7" t="s">
-        <v>155</v>
-      </c>
-      <c r="E7" t="s">
-        <v>156</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="G7" t="s">
-        <v>176</v>
       </c>
       <c r="H7">
         <v>13</v>
@@ -2919,22 +2934,22 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
+        <v>176</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" t="s">
+        <v>154</v>
+      </c>
+      <c r="E8" t="s">
+        <v>155</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="G8" t="s">
         <v>178</v>
-      </c>
-      <c r="D8" t="s">
-        <v>155</v>
-      </c>
-      <c r="E8" t="s">
-        <v>156</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="G8" t="s">
-        <v>179</v>
       </c>
       <c r="H8">
         <v>38</v>
@@ -2951,22 +2966,22 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
+        <v>179</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" t="s">
+        <v>154</v>
+      </c>
+      <c r="E9" t="s">
+        <v>155</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="G9" t="s">
         <v>181</v>
-      </c>
-      <c r="D9" t="s">
-        <v>155</v>
-      </c>
-      <c r="E9" t="s">
-        <v>156</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="G9" t="s">
-        <v>182</v>
       </c>
       <c r="H9">
         <v>9</v>
@@ -2986,22 +3001,22 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
+        <v>182</v>
+      </c>
+      <c r="C10" t="s">
         <v>183</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
+        <v>154</v>
+      </c>
+      <c r="E10" t="s">
+        <v>155</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="D10" t="s">
-        <v>155</v>
-      </c>
-      <c r="E10" t="s">
-        <v>156</v>
-      </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" t="s">
         <v>185</v>
-      </c>
-      <c r="G10" t="s">
-        <v>186</v>
       </c>
       <c r="H10">
         <v>0</v>
@@ -3018,22 +3033,22 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
+        <v>186</v>
+      </c>
+      <c r="C11" t="s">
         <v>187</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
+        <v>154</v>
+      </c>
+      <c r="E11" t="s">
+        <v>160</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="G11" t="s">
         <v>188</v>
-      </c>
-      <c r="D11" t="s">
-        <v>155</v>
-      </c>
-      <c r="E11" t="s">
-        <v>161</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="G11" t="s">
-        <v>189</v>
       </c>
       <c r="H11">
         <v>63</v>
@@ -3053,22 +3068,22 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
+        <v>189</v>
+      </c>
+      <c r="C12" t="s">
         <v>190</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
+        <v>154</v>
+      </c>
+      <c r="E12" t="s">
+        <v>160</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="G12" t="s">
         <v>191</v>
-      </c>
-      <c r="D12" t="s">
-        <v>155</v>
-      </c>
-      <c r="E12" t="s">
-        <v>161</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="G12" t="s">
-        <v>192</v>
       </c>
       <c r="H12">
         <v>65</v>
@@ -3082,22 +3097,22 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
+        <v>192</v>
+      </c>
+      <c r="C13" t="s">
         <v>193</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
+        <v>154</v>
+      </c>
+      <c r="E13" t="s">
+        <v>155</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="G13" t="s">
         <v>194</v>
-      </c>
-      <c r="D13" t="s">
-        <v>155</v>
-      </c>
-      <c r="E13" t="s">
-        <v>156</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="G13" t="s">
-        <v>195</v>
       </c>
       <c r="H13">
         <v>14</v>

</xml_diff>